<commit_message>
more specific carriers for loads
</commit_message>
<xml_diff>
--- a/data/loads.xlsx
+++ b/data/loads.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Keks-repo\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E47209F-4D8E-4493-AE20-A5E10C7CE055}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21F58A21-E846-4CE5-8FA0-6B52D3C34797}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="21570" windowHeight="9180" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="32">
   <si>
     <t>name</t>
   </si>
@@ -40,9 +40,6 @@
     <t>Industry_1</t>
   </si>
   <si>
-    <t>AC</t>
-  </si>
-  <si>
     <t>kritis</t>
   </si>
   <si>
@@ -61,9 +58,6 @@
     <t>Industry_1_HT</t>
   </si>
   <si>
-    <t>thermal</t>
-  </si>
-  <si>
     <t>kritis_thermal</t>
   </si>
   <si>
@@ -110,6 +104,18 @@
   </si>
   <si>
     <t>Residential_3_LT</t>
+  </si>
+  <si>
+    <t>industry_AC</t>
+  </si>
+  <si>
+    <t>kritis_AC</t>
+  </si>
+  <si>
+    <t>residential_AC</t>
+  </si>
+  <si>
+    <t>residential_thermal</t>
   </si>
 </sst>
 </file>
@@ -453,6 +459,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="16.42578125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -477,7 +484,7 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>28</v>
       </c>
       <c r="D2">
         <v>5.6959999999999997E-2</v>
@@ -485,13 +492,13 @@
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>6</v>
+      </c>
+      <c r="B3" t="s">
         <v>7</v>
       </c>
-      <c r="B3" t="s">
-        <v>8</v>
-      </c>
       <c r="C3" t="s">
-        <v>6</v>
+        <v>29</v>
       </c>
       <c r="D3">
         <v>6.0600000000000003E-3</v>
@@ -499,13 +506,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>8</v>
+      </c>
+      <c r="B4" t="s">
         <v>9</v>
       </c>
-      <c r="B4" t="s">
-        <v>10</v>
-      </c>
       <c r="C4" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="D4">
         <v>6.6689999999999999E-2</v>
@@ -513,13 +520,13 @@
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
         <v>11</v>
       </c>
-      <c r="B5" t="s">
-        <v>12</v>
-      </c>
       <c r="C5" t="s">
-        <v>13</v>
+        <v>10</v>
       </c>
       <c r="D5">
         <v>0.17510999999999999</v>
@@ -527,13 +534,13 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B6" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="D6">
         <v>4.1880000000000001E-2</v>
@@ -541,13 +548,13 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B7" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="C7" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D7">
         <v>2.1112899999999999</v>
@@ -555,13 +562,13 @@
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B8" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="C8" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="D8">
         <v>2.001E-2</v>
@@ -569,13 +576,13 @@
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B9" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="C9" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D9">
         <v>2.111E-2</v>
@@ -583,13 +590,13 @@
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B10" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="C10" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D10">
         <v>0.63175000000000003</v>
@@ -597,13 +604,13 @@
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C11" t="s">
-        <v>6</v>
+        <v>30</v>
       </c>
       <c r="D11">
         <v>3.3340000000000002E-2</v>
@@ -611,13 +618,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="C12" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D12">
         <v>3.5180000000000003E-2</v>
@@ -625,13 +632,13 @@
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B13" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="C13" t="s">
-        <v>13</v>
+        <v>31</v>
       </c>
       <c r="D13">
         <v>1.05291</v>

</xml_diff>